<commit_message>
#52 Client BOM Update With Peripherals.
</commit_message>
<xml_diff>
--- a/Design Files/Stepper-Driver-v2.0/BOM/Client-BOM-Stepper-Driver-v2.0.xlsx
+++ b/Design Files/Stepper-Driver-v2.0/BOM/Client-BOM-Stepper-Driver-v2.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\muhunthancanagey-servocontrol\Design Files\Stepper-Driver-v2.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="397">
   <si>
     <t>#</t>
   </si>
@@ -30,6 +30,9 @@
     <t>Capacitor</t>
   </si>
   <si>
+    <t>Capacitors</t>
+  </si>
+  <si>
     <t>Diode</t>
   </si>
   <si>
@@ -117,6 +120,9 @@
     <t>C6, C8, C18, C52, C53, C54, C55, C57, C59, C68, C69, C70, C71, C73, C75</t>
   </si>
   <si>
+    <t>C7, C9, C16</t>
+  </si>
+  <si>
     <t>C10, C19, C20</t>
   </si>
   <si>
@@ -144,6 +150,9 @@
     <t>C32, C33, C34, C35</t>
   </si>
   <si>
+    <t>C46, C47, C56, C58, C62, C63, C72, C74, C78</t>
+  </si>
+  <si>
     <t>C48, C49, C50, C51, C64, C65, C66, C67</t>
   </si>
   <si>
@@ -234,7 +243,7 @@
     <t>Q3</t>
   </si>
   <si>
-    <t>R1</t>
+    <t>R1, R4, R5</t>
   </si>
   <si>
     <t>R2</t>
@@ -243,9 +252,6 @@
     <t>R3</t>
   </si>
   <si>
-    <t>R4, R5</t>
-  </si>
-  <si>
     <t>R6</t>
   </si>
   <si>
@@ -360,6 +366,9 @@
     <t>CAP CER 1UF 50V X5R 0603</t>
   </si>
   <si>
+    <t>CAP CER 0.1UF 50V X7R 0603</t>
+  </si>
+  <si>
     <t>CAP CER 4.7UF 50V X7R 1206</t>
   </si>
   <si>
@@ -390,7 +399,7 @@
     <t>CAP CER 0.1UF 50V X7R 0402</t>
   </si>
   <si>
-    <t>100uF 50V ±20% SMD,D6.3xL7.7mm Aluminum Electrolytic Capacitors - SMD ROHS</t>
+    <t>35V 100uF Polymer ±20% SMD,D6.3xL9mm Polymer Aluminum Capacitors ROHS</t>
   </si>
   <si>
     <t>CAP CER 1000PF 25V C0G 0402</t>
@@ -480,7 +489,7 @@
     <t>40V 200mW 100 200mA NPN SOT-23 Bipolar (BJT) ROHS</t>
   </si>
   <si>
-    <t>RES 100K OHM 1% 1/8W 0805</t>
+    <t>RES SMD 100K OHM 0.1% 1/16W 0402</t>
   </si>
   <si>
     <t>RES 3.9K OHM 1% 1/16W 0402</t>
@@ -489,9 +498,6 @@
     <t>RES SMD 698K OHM 0.1% 1/8W 0805</t>
   </si>
   <si>
-    <t>RES SMD 100K OHM 0.1% 1/16W 0402</t>
-  </si>
-  <si>
     <t>RES SMD 51.1K OHM 0.1% 1/8W 0805</t>
   </si>
   <si>
@@ -612,7 +618,7 @@
     <t>cap-0402</t>
   </si>
   <si>
-    <t>RVT1H101M0607</t>
+    <t>SVZ1VM101E09E00RAXXX</t>
   </si>
   <si>
     <t>SMB_</t>
@@ -648,9 +654,6 @@
     <t>HDR1X3_</t>
   </si>
   <si>
-    <t>TC2030-IDC_</t>
-  </si>
-  <si>
     <t>U263-163N-4BQC65</t>
   </si>
   <si>
@@ -678,12 +681,12 @@
     <t>Sot-23</t>
   </si>
   <si>
+    <t>Res-0402</t>
+  </si>
+  <si>
     <t>RES-0805</t>
   </si>
   <si>
-    <t>Res-0402</t>
-  </si>
-  <si>
     <t>Res-0603</t>
   </si>
   <si>
@@ -840,7 +843,7 @@
     <t>MMBT3904</t>
   </si>
   <si>
-    <t>RC0805FR-07100KL</t>
+    <t>RT0402BRD07100KL</t>
   </si>
   <si>
     <t>RC0402FR-073K9L</t>
@@ -849,9 +852,6 @@
     <t>RT0805BRD07698KL</t>
   </si>
   <si>
-    <t>RT0402BRD07100KL</t>
-  </si>
-  <si>
     <t>RT0805BRD0751K1L</t>
   </si>
   <si>
@@ -966,6 +966,9 @@
     <t>TDK</t>
   </si>
   <si>
+    <t>KNSCHA</t>
+  </si>
+  <si>
     <t>Diodes</t>
   </si>
   <si>
@@ -1152,15 +1155,12 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>Value</t>
+  </si>
+  <si>
     <t>Remarks</t>
   </si>
   <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>C7, C9, C16, C46, C47, C56, C58, C62, C63, C72, C74, C78</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -1168,13 +1168,55 @@
   </si>
   <si>
     <t>Tag Connect</t>
+  </si>
+  <si>
+    <t>Qty: 2 cables per whole order</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>Fuse</t>
+  </si>
+  <si>
+    <t>Shunt Jumper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stepper Motor </t>
+  </si>
+  <si>
+    <t>DO NOT MOUNT</t>
+  </si>
+  <si>
+    <t>Tag Connect Cable</t>
+  </si>
+  <si>
+    <t>X2541-A1NIB</t>
+  </si>
+  <si>
+    <t>Open top 3A 2.54mm P=2.54mm Shunts, Jumpers ROHS</t>
+  </si>
+  <si>
+    <t>028707.5PXCN</t>
+  </si>
+  <si>
+    <t>32V Blade fuse 7.5A Automotive Fuses ROHS</t>
+  </si>
+  <si>
+    <t>Should be provided by Client</t>
+  </si>
+  <si>
+    <t>TC2030-CTX 6-Pin Cable for ARM Cortex ATMEL</t>
+  </si>
+  <si>
+    <t>TC2030-CTX</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1213,6 +1255,30 @@
     <font>
       <b/>
       <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1333,7 +1399,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1368,6 +1434,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1660,19 +1744,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.42578125" customWidth="1"/>
+    <col min="11" max="11" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1684,9 +1768,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1697,16 +1781,16 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>307</v>
@@ -1715,10 +1799,10 @@
         <v>378</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1731,22 +1815,22 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H3" s="7" t="s">
         <v>308</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="J3" s="7">
         <v>2</v>
@@ -1756,29 +1840,29 @@
     <row r="4" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B83" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B84" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>381</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>309</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
@@ -1791,26 +1875,26 @@
         <f>ROW(B5) - ROW($B$2)</f>
         <v>3</v>
       </c>
-      <c r="C5" s="13" t="s">
-        <v>2</v>
+      <c r="C5" s="12" t="s">
+        <v>3</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H5" s="7" t="s">
         <v>310</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -1823,26 +1907,26 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C6" s="13" t="s">
-        <v>2</v>
+      <c r="C6" s="12" t="s">
+        <v>3</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>311</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1859,29 +1943,29 @@
         <v>2</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="H7" s="7" t="s">
         <v>312</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="J7" s="7">
         <v>15</v>
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -1891,25 +1975,25 @@
         <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>379</v>
+        <v>33</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>314</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="J8" s="9">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="K8" s="9"/>
     </row>
@@ -1923,22 +2007,22 @@
         <v>2</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H9" s="7" t="s">
         <v>313</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J9" s="7">
         <v>3</v>
@@ -1955,22 +2039,22 @@
         <v>2</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>310</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J10" s="9">
         <v>2</v>
@@ -1987,22 +2071,22 @@
         <v>2</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>311</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J11" s="7">
         <v>3</v>
@@ -2019,22 +2103,22 @@
         <v>2</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>310</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -2051,22 +2135,22 @@
         <v>2</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="H13" s="7" t="s">
         <v>311</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
@@ -2083,22 +2167,22 @@
         <v>2</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>310</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J14" s="9">
         <v>3</v>
@@ -2115,22 +2199,22 @@
         <v>2</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>310</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J15" s="7">
         <v>14</v>
@@ -2147,22 +2231,22 @@
         <v>2</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>310</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="J16" s="9">
         <v>2</v>
@@ -2179,2137 +2263,2269 @@
         <v>2</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>310</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J17" s="7">
         <v>4</v>
       </c>
       <c r="K17" s="7"/>
     </row>
-    <row r="18" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
-        <f>ROW(B18) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>123</v>
+      <c r="D18" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>125</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>381</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="I18" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="I18" s="10" t="s">
         <v>352</v>
       </c>
-      <c r="J18" s="7">
-        <v>8</v>
-      </c>
-      <c r="K18" s="7"/>
-    </row>
-    <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J18" s="9">
+        <v>9</v>
+      </c>
+      <c r="K18" s="9"/>
+    </row>
+    <row r="19" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B19) - ROW($B$2)</f>
         <v>17</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>124</v>
+      <c r="D19" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>126</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>251</v>
-      </c>
-      <c r="H19" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="I19" s="10" t="s">
+        <v>381</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="I19" s="8" t="s">
         <v>353</v>
       </c>
-      <c r="J19" s="9">
-        <v>4</v>
-      </c>
-      <c r="K19" s="9"/>
+      <c r="J19" s="7">
+        <v>8</v>
+      </c>
+      <c r="K19" s="7"/>
     </row>
     <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
-        <f>ROW(B20) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C20" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="G20" s="8" t="s">
+      <c r="C20" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="G20" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="H20" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="I20" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J20" s="7">
-        <v>1</v>
-      </c>
-      <c r="K20" s="7"/>
-    </row>
-    <row r="21" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H20" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="I20" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="J20" s="9">
+        <v>4</v>
+      </c>
+      <c r="K20" s="9"/>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B21) - ROW($B$2)</f>
         <v>19</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="D21" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="G21" s="10" t="s">
+      <c r="D21" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="G21" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="H21" s="7" t="s">
         <v>316</v>
       </c>
       <c r="I21" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J21" s="9">
-        <v>1</v>
-      </c>
-      <c r="K21" s="9"/>
-    </row>
-    <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J21" s="7">
+        <v>1</v>
+      </c>
+      <c r="K21" s="7"/>
+    </row>
+    <row r="22" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
-        <f>ROW(B22) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="G22" s="8" t="s">
+      <c r="D22" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="G22" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="H22" s="7" t="s">
-        <v>315</v>
+      <c r="H22" s="9" t="s">
+        <v>317</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J22" s="7">
-        <v>1</v>
-      </c>
-      <c r="K22" s="7"/>
-    </row>
-    <row r="23" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J22" s="9">
+        <v>1</v>
+      </c>
+      <c r="K22" s="9"/>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B23) - ROW($B$2)</f>
         <v>21</v>
       </c>
-      <c r="C23" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="G23" s="10" t="s">
+      <c r="C23" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="G23" s="8" t="s">
         <v>255</v>
       </c>
-      <c r="H23" s="9" t="s">
+      <c r="H23" s="7" t="s">
         <v>316</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J23" s="9">
-        <v>1</v>
-      </c>
-      <c r="K23" s="9"/>
-    </row>
-    <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J23" s="7">
+        <v>1</v>
+      </c>
+      <c r="K23" s="7"/>
+    </row>
+    <row r="24" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
-        <f>ROW(B24) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C24" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="G24" s="8" t="s">
+      <c r="C24" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="G24" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="H24" s="7" t="s">
+      <c r="H24" s="9" t="s">
         <v>317</v>
       </c>
       <c r="I24" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J24" s="7">
-        <v>1</v>
-      </c>
-      <c r="K24" s="7"/>
+      <c r="J24" s="9">
+        <v>1</v>
+      </c>
+      <c r="K24" s="9"/>
     </row>
     <row r="25" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B25) - ROW($B$2)</f>
         <v>23</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="D25" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="E25" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>200</v>
-      </c>
-      <c r="G25" s="10" t="s">
+      <c r="D25" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="G25" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="H25" s="7" t="s">
         <v>318</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J25" s="9">
-        <v>4</v>
-      </c>
-      <c r="K25" s="9"/>
+      <c r="J25" s="7">
+        <v>1</v>
+      </c>
+      <c r="K25" s="7"/>
     </row>
     <row r="26" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
-        <f>ROW(B26) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C26" s="12" t="s">
+      <c r="C26" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D26" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="G26" s="8" t="s">
+      <c r="D26" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="G26" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="H26" s="7" t="s">
+      <c r="H26" s="9" t="s">
         <v>319</v>
       </c>
       <c r="I26" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J26" s="7">
-        <v>1</v>
-      </c>
-      <c r="K26" s="7"/>
+      <c r="J26" s="9">
+        <v>4</v>
+      </c>
+      <c r="K26" s="9"/>
     </row>
     <row r="27" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B27) - ROW($B$2)</f>
         <v>25</v>
       </c>
-      <c r="C27" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>202</v>
-      </c>
-      <c r="G27" s="10" t="s">
+      <c r="C27" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="G27" s="8" t="s">
         <v>259</v>
       </c>
-      <c r="H27" s="9" t="s">
-        <v>319</v>
+      <c r="H27" s="7" t="s">
+        <v>320</v>
       </c>
       <c r="I27" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J27" s="9">
-        <v>1</v>
-      </c>
-      <c r="K27" s="9"/>
+      <c r="J27" s="7">
+        <v>1</v>
+      </c>
+      <c r="K27" s="7"/>
     </row>
     <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
-        <f>ROW(B28) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C28" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="F28" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="G28" s="8" t="s">
+      <c r="C28" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="G28" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="H28" s="7" t="s">
+      <c r="H28" s="9" t="s">
         <v>320</v>
       </c>
       <c r="I28" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J28" s="7">
-        <v>1</v>
-      </c>
-      <c r="K28" s="7"/>
+      <c r="J28" s="9">
+        <v>1</v>
+      </c>
+      <c r="K28" s="9"/>
     </row>
     <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B29) - ROW($B$2)</f>
         <v>27</v>
       </c>
-      <c r="C29" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="D29" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="E29" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="F29" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="G29" s="10" t="s">
+      <c r="C29" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="G29" s="8" t="s">
         <v>261</v>
       </c>
-      <c r="H29" s="9" t="s">
+      <c r="H29" s="7" t="s">
         <v>321</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J29" s="9">
-        <v>1</v>
-      </c>
-      <c r="K29" s="9"/>
+      <c r="J29" s="7">
+        <v>1</v>
+      </c>
+      <c r="K29" s="7"/>
     </row>
     <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
-        <f>ROW(B30) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C30" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>204</v>
-      </c>
-      <c r="G30" s="8" t="s">
+      <c r="C30" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="G30" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="H30" s="7" t="s">
+      <c r="H30" s="9" t="s">
         <v>322</v>
       </c>
       <c r="I30" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J30" s="7">
-        <v>1</v>
-      </c>
-      <c r="K30" s="7"/>
+      <c r="J30" s="9">
+        <v>1</v>
+      </c>
+      <c r="K30" s="9"/>
     </row>
     <row r="31" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B31) - ROW($B$2)</f>
         <v>29</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D31" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="G31" s="10" t="s">
+      <c r="D31" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="G31" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="H31" s="9" t="s">
-        <v>311</v>
+      <c r="H31" s="7" t="s">
+        <v>323</v>
       </c>
       <c r="I31" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J31" s="9">
-        <v>1</v>
-      </c>
-      <c r="K31" s="9"/>
+      <c r="J31" s="7">
+        <v>1</v>
+      </c>
+      <c r="K31" s="7"/>
     </row>
     <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
-        <f>ROW(B32) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C32" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D32" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>137</v>
+      <c r="D32" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>139</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>381</v>
-      </c>
-      <c r="G32" s="8" t="s">
-        <v>206</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>323</v>
+        <v>207</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>311</v>
       </c>
       <c r="I32" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J32" s="7">
-        <v>1</v>
-      </c>
-      <c r="K32" s="7"/>
-    </row>
-    <row r="33" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J32" s="9">
+        <v>1</v>
+      </c>
+      <c r="K32" s="9"/>
+    </row>
+    <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B33) - ROW($B$2)</f>
         <v>31</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D33" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>138</v>
+      <c r="D33" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>140</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>381</v>
       </c>
-      <c r="G33" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="H33" s="9" t="s">
+      <c r="G33" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="H33" s="7" t="s">
         <v>324</v>
       </c>
       <c r="I33" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J33" s="9">
-        <v>1</v>
-      </c>
-      <c r="K33" s="9"/>
+      <c r="J33" s="7">
+        <v>1</v>
+      </c>
+      <c r="K33" s="7"/>
     </row>
     <row r="34" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
-        <f>ROW(B34) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="C34" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D34" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="F34" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="G34" s="8" t="s">
-        <v>264</v>
-      </c>
-      <c r="H34" s="7" t="s">
+      <c r="D34" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="G34" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="H34" s="9" t="s">
         <v>325</v>
       </c>
       <c r="I34" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J34" s="7">
-        <v>1</v>
-      </c>
-      <c r="K34" s="7"/>
-    </row>
-    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J34" s="9">
+        <v>1</v>
+      </c>
+      <c r="K34" s="9"/>
+    </row>
+    <row r="35" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B35) - ROW($B$2)</f>
         <v>33</v>
       </c>
-      <c r="C35" s="13" t="s">
-        <v>382</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="E35" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>209</v>
-      </c>
-      <c r="G35" s="10" t="s">
+      <c r="C35" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="G35" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="H35" s="9" t="s">
+      <c r="H35" s="7" t="s">
         <v>326</v>
       </c>
       <c r="I35" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J35" s="9">
-        <v>1</v>
-      </c>
-      <c r="K35" s="9"/>
-    </row>
-    <row r="36" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J35" s="7">
+        <v>1</v>
+      </c>
+      <c r="K35" s="7"/>
+    </row>
+    <row r="36" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="11">
-        <f>ROW(B36) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C36" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="D36" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="F36" s="9" t="s">
+      <c r="C36" s="15" t="s">
+        <v>382</v>
+      </c>
+      <c r="D36" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="F36" s="16" t="s">
         <v>381</v>
       </c>
-      <c r="G36" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="H36" s="7" t="s">
+      <c r="G36" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="H36" s="16" t="s">
         <v>327</v>
       </c>
-      <c r="I36" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J36" s="7">
-        <v>1</v>
-      </c>
-      <c r="K36" s="7"/>
-    </row>
-    <row r="37" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I36" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="J36" s="16">
+        <v>1</v>
+      </c>
+      <c r="K36" s="14" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B37) - ROW($B$2)</f>
         <v>35</v>
       </c>
-      <c r="C37" s="13" t="s">
+      <c r="C37" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="D37" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="E37" s="10" t="s">
-        <v>142</v>
+      <c r="D37" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>144</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>381</v>
       </c>
-      <c r="G37" s="10" t="s">
+      <c r="G37" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="H37" s="9" t="s">
+      <c r="H37" s="7" t="s">
         <v>328</v>
       </c>
       <c r="I37" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J37" s="9">
-        <v>1</v>
-      </c>
-      <c r="K37" s="9"/>
-    </row>
-    <row r="38" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J37" s="7">
+        <v>1</v>
+      </c>
+      <c r="K37" s="7"/>
+    </row>
+    <row r="38" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="11">
-        <f>ROW(B38) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C38" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="F38" s="7" t="s">
+      <c r="C38" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="F38" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="G38" s="10" t="s">
         <v>212</v>
       </c>
-      <c r="G38" s="8" t="s">
-        <v>266</v>
-      </c>
-      <c r="H38" s="7" t="s">
-        <v>325</v>
+      <c r="H38" s="9" t="s">
+        <v>329</v>
       </c>
       <c r="I38" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J38" s="7">
-        <v>2</v>
-      </c>
-      <c r="K38" s="7"/>
+      <c r="J38" s="9">
+        <v>1</v>
+      </c>
+      <c r="K38" s="9"/>
     </row>
     <row r="39" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B39) - ROW($B$2)</f>
         <v>37</v>
       </c>
-      <c r="C39" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D39" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="E39" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="F39" s="9" t="s">
-        <v>381</v>
-      </c>
-      <c r="G39" s="10" t="s">
+      <c r="C39" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="F39" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="H39" s="9" t="s">
-        <v>324</v>
+      <c r="G39" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>326</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="J39" s="9">
-        <v>4</v>
-      </c>
-      <c r="K39" s="9"/>
-    </row>
-    <row r="40" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J39" s="7">
+        <v>2</v>
+      </c>
+      <c r="K39" s="7"/>
+    </row>
+    <row r="40" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="11">
-        <f>ROW(B40) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C40" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>145</v>
+      <c r="C40" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>147</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>381</v>
       </c>
-      <c r="G40" s="8" t="s">
+      <c r="G40" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="H40" s="7" t="s">
-        <v>320</v>
+      <c r="H40" s="9" t="s">
+        <v>325</v>
       </c>
       <c r="I40" s="8" t="s">
-        <v>354</v>
-      </c>
-      <c r="J40" s="7">
-        <v>1</v>
-      </c>
-      <c r="K40" s="7"/>
-    </row>
-    <row r="41" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>380</v>
+      </c>
+      <c r="J40" s="9">
+        <v>4</v>
+      </c>
+      <c r="K40" s="9"/>
+    </row>
+    <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B41) - ROW($B$2)</f>
         <v>39</v>
       </c>
-      <c r="C41" s="13" t="s">
+      <c r="C41" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D41" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="E41" s="10" t="s">
-        <v>146</v>
+      <c r="D41" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>148</v>
       </c>
       <c r="F41" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="G41" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="G41" s="10" t="s">
-        <v>267</v>
-      </c>
-      <c r="H41" s="9" t="s">
-        <v>329</v>
-      </c>
-      <c r="I41" s="10" t="s">
-        <v>380</v>
-      </c>
-      <c r="J41" s="9">
-        <v>8</v>
-      </c>
-      <c r="K41" s="9"/>
+      <c r="H41" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="I41" s="8" t="s">
+        <v>355</v>
+      </c>
+      <c r="J41" s="7">
+        <v>1</v>
+      </c>
+      <c r="K41" s="7"/>
     </row>
     <row r="42" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="11">
-        <f>ROW(B42) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C42" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D42" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="G42" s="8" t="s">
+      <c r="C42" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E42" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="G42" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="H42" s="7" t="s">
-        <v>329</v>
+      <c r="H42" s="9" t="s">
+        <v>330</v>
       </c>
       <c r="I42" s="10" t="s">
         <v>380</v>
       </c>
-      <c r="J42" s="7">
-        <v>1</v>
-      </c>
-      <c r="K42" s="7"/>
-    </row>
-    <row r="43" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J42" s="9">
+        <v>8</v>
+      </c>
+      <c r="K42" s="9"/>
+    </row>
+    <row r="43" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B43) - ROW($B$2)</f>
         <v>41</v>
       </c>
-      <c r="C43" s="13" t="s">
+      <c r="C43" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="D43" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="E43" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="F43" s="9" t="s">
-        <v>381</v>
-      </c>
-      <c r="G43" s="10" t="s">
+      <c r="D43" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="F43" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="H43" s="9" t="s">
+      <c r="G43" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="H43" s="7" t="s">
         <v>330</v>
       </c>
       <c r="I43" s="10" t="s">
         <v>380</v>
       </c>
-      <c r="J43" s="9">
-        <v>5</v>
-      </c>
-      <c r="K43" s="9"/>
-    </row>
-    <row r="44" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J43" s="7">
+        <v>1</v>
+      </c>
+      <c r="K43" s="7"/>
+    </row>
+    <row r="44" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="11">
-        <f>ROW(B44) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="C44" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="E44" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="G44" s="8" t="s">
-        <v>269</v>
-      </c>
-      <c r="H44" s="7" t="s">
+      <c r="C44" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E44" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="G44" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="H44" s="9" t="s">
         <v>331</v>
       </c>
       <c r="I44" s="10" t="s">
         <v>380</v>
       </c>
-      <c r="J44" s="7">
-        <v>4</v>
-      </c>
-      <c r="K44" s="7"/>
-    </row>
-    <row r="45" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J44" s="9">
+        <v>5</v>
+      </c>
+      <c r="K44" s="9"/>
+    </row>
+    <row r="45" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B45) - ROW($B$2)</f>
         <v>43</v>
       </c>
-      <c r="C45" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D45" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E45" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="F45" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="G45" s="10" t="s">
+      <c r="C45" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E45" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="G45" s="8" t="s">
         <v>270</v>
       </c>
-      <c r="H45" s="9" t="s">
+      <c r="H45" s="7" t="s">
         <v>332</v>
       </c>
       <c r="I45" s="10" t="s">
         <v>380</v>
       </c>
-      <c r="J45" s="9">
-        <v>1</v>
-      </c>
-      <c r="K45" s="9"/>
+      <c r="J45" s="7">
+        <v>4</v>
+      </c>
+      <c r="K45" s="7"/>
     </row>
     <row r="46" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="11">
-        <f>ROW(B46) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="C46" s="12" t="s">
+      <c r="C46" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D46" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="E46" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="F46" s="7" t="s">
+      <c r="D46" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E46" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="F46" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="G46" s="8" t="s">
+      <c r="G46" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="H46" s="7" t="s">
-        <v>321</v>
+      <c r="H46" s="9" t="s">
+        <v>333</v>
       </c>
       <c r="I46" s="10" t="s">
         <v>380</v>
       </c>
-      <c r="J46" s="7">
-        <v>1</v>
-      </c>
-      <c r="K46" s="7"/>
-    </row>
-    <row r="47" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J46" s="9">
+        <v>1</v>
+      </c>
+      <c r="K46" s="9"/>
+    </row>
+    <row r="47" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B47) - ROW($B$2)</f>
         <v>45</v>
       </c>
-      <c r="C47" s="13" t="s">
+      <c r="C47" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D47" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E47" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="F47" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="G47" s="10" t="s">
+      <c r="D47" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="G47" s="8" t="s">
         <v>272</v>
       </c>
-      <c r="H47" s="9" t="s">
-        <v>333</v>
+      <c r="H47" s="7" t="s">
+        <v>322</v>
       </c>
       <c r="I47" s="10" t="s">
         <v>380</v>
       </c>
-      <c r="J47" s="9">
-        <v>1</v>
-      </c>
-      <c r="K47" s="9"/>
-    </row>
-    <row r="48" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J47" s="7">
+        <v>1</v>
+      </c>
+      <c r="K47" s="7"/>
+    </row>
+    <row r="48" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="11">
-        <f>ROW(B48) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="C48" s="12" t="s">
+      <c r="C48" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D48" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E48" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="F48" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="G48" s="8" t="s">
+      <c r="D48" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E48" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="F48" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="G48" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="H48" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="I48" s="8" t="s">
-        <v>355</v>
-      </c>
-      <c r="J48" s="7">
-        <v>1</v>
-      </c>
-      <c r="K48" s="7"/>
+      <c r="H48" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="I48" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J48" s="9">
+        <v>1</v>
+      </c>
+      <c r="K48" s="9"/>
     </row>
     <row r="49" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B49) - ROW($B$2)</f>
         <v>47</v>
       </c>
-      <c r="C49" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D49" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="F49" s="9" t="s">
+      <c r="C49" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E49" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="F49" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="G49" s="10" t="s">
+      <c r="G49" s="8" t="s">
         <v>274</v>
       </c>
-      <c r="H49" s="9" t="s">
+      <c r="H49" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="I49" s="10" t="s">
+      <c r="I49" s="8" t="s">
         <v>356</v>
       </c>
-      <c r="J49" s="9">
-        <v>1</v>
-      </c>
-      <c r="K49" s="9"/>
+      <c r="J49" s="7">
+        <v>3</v>
+      </c>
+      <c r="K49" s="7"/>
     </row>
     <row r="50" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="11">
-        <f>ROW(B50) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="C50" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D50" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E50" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="G50" s="8" t="s">
+      <c r="C50" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E50" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="G50" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="H50" s="7" t="s">
+      <c r="H50" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="I50" s="8" t="s">
+      <c r="I50" s="10" t="s">
         <v>357</v>
       </c>
-      <c r="J50" s="7">
-        <v>1</v>
-      </c>
-      <c r="K50" s="7"/>
+      <c r="J50" s="9">
+        <v>1</v>
+      </c>
+      <c r="K50" s="9"/>
     </row>
     <row r="51" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B51) - ROW($B$2)</f>
         <v>49</v>
       </c>
-      <c r="C51" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D51" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="E51" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>220</v>
-      </c>
-      <c r="G51" s="10" t="s">
+      <c r="C51" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="G51" s="8" t="s">
         <v>276</v>
       </c>
-      <c r="H51" s="9" t="s">
+      <c r="H51" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="I51" s="10" t="s">
-        <v>355</v>
-      </c>
-      <c r="J51" s="9">
-        <v>2</v>
-      </c>
-      <c r="K51" s="9"/>
+      <c r="I51" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="J51" s="7">
+        <v>1</v>
+      </c>
+      <c r="K51" s="7"/>
     </row>
     <row r="52" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="11">
-        <f>ROW(B52) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="C52" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D52" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E52" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F52" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="G52" s="8" t="s">
+      <c r="C52" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="E52" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="G52" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="H52" s="7" t="s">
+      <c r="H52" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="I52" s="8" t="s">
-        <v>358</v>
-      </c>
-      <c r="J52" s="7">
-        <v>1</v>
-      </c>
-      <c r="K52" s="7"/>
+      <c r="I52" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="J52" s="9">
+        <v>1</v>
+      </c>
+      <c r="K52" s="9"/>
     </row>
     <row r="53" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B53) - ROW($B$2)</f>
         <v>51</v>
       </c>
-      <c r="C53" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="D53" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="E53" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="F53" s="9" t="s">
+      <c r="C53" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="E53" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="F53" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="G53" s="10" t="s">
+      <c r="G53" s="8" t="s">
         <v>278</v>
       </c>
-      <c r="H53" s="9" t="s">
+      <c r="H53" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="I53" s="10" t="s">
-        <v>359</v>
-      </c>
-      <c r="J53" s="9">
-        <v>1</v>
-      </c>
-      <c r="K53" s="9"/>
+      <c r="I53" s="8" t="s">
+        <v>360</v>
+      </c>
+      <c r="J53" s="7">
+        <v>1</v>
+      </c>
+      <c r="K53" s="7"/>
     </row>
     <row r="54" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="11">
-        <f>ROW(B54) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="C54" s="12"/>
-      <c r="D54" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="E54" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="F54" s="7" t="s">
+      <c r="C54" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E54" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="F54" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="G54" s="8" t="s">
+      <c r="G54" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="H54" s="7" t="s">
+      <c r="H54" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="I54" s="8" t="s">
-        <v>360</v>
-      </c>
-      <c r="J54" s="7">
-        <v>1</v>
-      </c>
-      <c r="K54" s="7"/>
+      <c r="I54" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="J54" s="9">
+        <v>1</v>
+      </c>
+      <c r="K54" s="9"/>
     </row>
     <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B55) - ROW($B$2)</f>
         <v>53</v>
       </c>
-      <c r="C55" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="D55" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="E55" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="F55" s="9" t="s">
+      <c r="C55" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E55" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="F55" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="G55" s="10" t="s">
+      <c r="G55" s="8" t="s">
         <v>280</v>
       </c>
-      <c r="H55" s="9" t="s">
+      <c r="H55" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="I55" s="10" t="s">
-        <v>361</v>
-      </c>
-      <c r="J55" s="9">
+      <c r="I55" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="J55" s="7">
         <v>3</v>
       </c>
-      <c r="K55" s="9"/>
+      <c r="K55" s="7"/>
     </row>
     <row r="56" spans="1:11" ht="96.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="11">
-        <f>ROW(B56) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="C56" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="E56" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="F56" s="7" t="s">
+      <c r="C56" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E56" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="F56" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="G56" s="8" t="s">
+      <c r="G56" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="H56" s="7" t="s">
+      <c r="H56" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="I56" s="8" t="s">
-        <v>362</v>
-      </c>
-      <c r="J56" s="7">
+      <c r="I56" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="J56" s="9">
         <v>67</v>
       </c>
-      <c r="K56" s="7"/>
+      <c r="K56" s="9"/>
     </row>
     <row r="57" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B57) - ROW($B$2)</f>
         <v>55</v>
       </c>
-      <c r="C57" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D57" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="E57" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="F57" s="9" t="s">
+      <c r="C57" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="E57" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="F57" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="G57" s="10" t="s">
+      <c r="G57" s="8" t="s">
         <v>282</v>
       </c>
-      <c r="H57" s="9" t="s">
+      <c r="H57" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="I57" s="10" t="s">
-        <v>363</v>
-      </c>
-      <c r="J57" s="9">
+      <c r="I57" s="8" t="s">
+        <v>364</v>
+      </c>
+      <c r="J57" s="7">
         <v>14</v>
       </c>
-      <c r="K57" s="9"/>
+      <c r="K57" s="7"/>
     </row>
     <row r="58" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="11">
-        <f>ROW(B58) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="C58" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D58" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E58" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="F58" s="7" t="s">
+      <c r="C58" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="E58" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="F58" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="G58" s="8" t="s">
+      <c r="G58" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="H58" s="7" t="s">
+      <c r="H58" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="I58" s="8" t="s">
-        <v>364</v>
-      </c>
-      <c r="J58" s="7">
+      <c r="I58" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="J58" s="9">
         <v>5</v>
       </c>
-      <c r="K58" s="7"/>
+      <c r="K58" s="9"/>
     </row>
     <row r="59" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B59) - ROW($B$2)</f>
         <v>57</v>
       </c>
-      <c r="C59" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D59" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="E59" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="F59" s="9" t="s">
+      <c r="C59" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="E59" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F59" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="G59" s="10" t="s">
+      <c r="G59" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="H59" s="9" t="s">
+      <c r="H59" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="I59" s="10" t="s">
-        <v>365</v>
-      </c>
-      <c r="J59" s="9">
+      <c r="I59" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="J59" s="7">
         <v>3</v>
       </c>
-      <c r="K59" s="9"/>
+      <c r="K59" s="7"/>
     </row>
     <row r="60" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="11">
-        <f>ROW(B60) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="C60" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D60" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="E60" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="F60" s="7" t="s">
+      <c r="C60" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E60" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="F60" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="G60" s="8" t="s">
+      <c r="G60" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="H60" s="7" t="s">
+      <c r="H60" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="I60" s="8" t="s">
-        <v>366</v>
-      </c>
-      <c r="J60" s="7">
+      <c r="I60" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="J60" s="9">
         <v>3</v>
       </c>
-      <c r="K60" s="7"/>
+      <c r="K60" s="9"/>
     </row>
     <row r="61" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B61) - ROW($B$2)</f>
         <v>59</v>
       </c>
-      <c r="C61" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D61" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="E61" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="F61" s="9" t="s">
+      <c r="C61" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E61" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="F61" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="G61" s="10" t="s">
+      <c r="G61" s="8" t="s">
         <v>286</v>
       </c>
-      <c r="H61" s="9" t="s">
+      <c r="H61" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="I61" s="10" t="s">
-        <v>367</v>
-      </c>
-      <c r="J61" s="9">
-        <v>1</v>
-      </c>
-      <c r="K61" s="9"/>
+      <c r="I61" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="J61" s="7">
+        <v>1</v>
+      </c>
+      <c r="K61" s="7"/>
     </row>
     <row r="62" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="11">
-        <f>ROW(B62) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="C62" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D62" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E62" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="F62" s="7" t="s">
+      <c r="C62" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E62" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="F62" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="G62" s="8" t="s">
+      <c r="G62" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="H62" s="7" t="s">
+      <c r="H62" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="I62" s="8" t="s">
-        <v>368</v>
-      </c>
-      <c r="J62" s="7">
-        <v>1</v>
-      </c>
-      <c r="K62" s="7"/>
+      <c r="I62" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="J62" s="9">
+        <v>1</v>
+      </c>
+      <c r="K62" s="9"/>
     </row>
     <row r="63" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B63) - ROW($B$2)</f>
         <v>61</v>
       </c>
-      <c r="C63" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D63" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="E63" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="F63" s="9" t="s">
+      <c r="C63" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D63" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E63" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="F63" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="G63" s="10" t="s">
+      <c r="G63" s="8" t="s">
         <v>288</v>
       </c>
-      <c r="H63" s="9" t="s">
+      <c r="H63" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="I63" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="J63" s="9">
+      <c r="I63" s="8" t="s">
+        <v>370</v>
+      </c>
+      <c r="J63" s="7">
         <v>2</v>
       </c>
-      <c r="K63" s="9"/>
+      <c r="K63" s="7"/>
     </row>
     <row r="64" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="11">
-        <f>ROW(B64) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>62</v>
       </c>
-      <c r="C64" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D64" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="E64" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="F64" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="G64" s="8" t="s">
+      <c r="C64" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E64" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="F64" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="G64" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="H64" s="7" t="s">
+      <c r="H64" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="I64" s="8" t="s">
-        <v>370</v>
-      </c>
-      <c r="J64" s="7">
+      <c r="I64" s="10" t="s">
+        <v>371</v>
+      </c>
+      <c r="J64" s="9">
         <v>2</v>
       </c>
-      <c r="K64" s="7"/>
+      <c r="K64" s="9"/>
     </row>
     <row r="65" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B65) - ROW($B$2)</f>
         <v>63</v>
       </c>
-      <c r="C65" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D65" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="E65" s="10" t="s">
-        <v>170</v>
-      </c>
-      <c r="F65" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="G65" s="10" t="s">
+      <c r="C65" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D65" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E65" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="F65" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="G65" s="8" t="s">
         <v>290</v>
       </c>
-      <c r="H65" s="9" t="s">
-        <v>334</v>
-      </c>
-      <c r="I65" s="10" t="s">
-        <v>371</v>
-      </c>
-      <c r="J65" s="9">
+      <c r="H65" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="I65" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="J65" s="7">
         <v>8</v>
       </c>
-      <c r="K65" s="9"/>
+      <c r="K65" s="7"/>
     </row>
     <row r="66" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
       <c r="B66" s="11">
-        <f>ROW(B66) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>64</v>
       </c>
-      <c r="C66" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D66" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="E66" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="F66" s="7" t="s">
+      <c r="C66" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="E66" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="F66" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="G66" s="8" t="s">
+      <c r="G66" s="10" t="s">
         <v>291</v>
       </c>
-      <c r="H66" s="7" t="s">
+      <c r="H66" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="I66" s="8" t="s">
-        <v>372</v>
-      </c>
-      <c r="J66" s="7">
+      <c r="I66" s="10" t="s">
+        <v>373</v>
+      </c>
+      <c r="J66" s="9">
         <v>4</v>
       </c>
-      <c r="K66" s="7"/>
+      <c r="K66" s="9"/>
     </row>
     <row r="67" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B67) - ROW($B$2)</f>
         <v>65</v>
       </c>
-      <c r="C67" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D67" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="E67" s="10" t="s">
-        <v>172</v>
-      </c>
-      <c r="F67" s="9" t="s">
+      <c r="C67" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D67" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E67" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="F67" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="G67" s="10" t="s">
+      <c r="G67" s="8" t="s">
         <v>292</v>
       </c>
-      <c r="H67" s="9" t="s">
+      <c r="H67" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="I67" s="10" t="s">
-        <v>373</v>
-      </c>
-      <c r="J67" s="9">
+      <c r="I67" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="J67" s="7">
         <v>8</v>
       </c>
-      <c r="K67" s="9"/>
+      <c r="K67" s="7"/>
     </row>
     <row r="68" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="11">
-        <f>ROW(B68) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>66</v>
       </c>
-      <c r="C68" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D68" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="E68" s="8" t="s">
-        <v>173</v>
+      <c r="C68" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D68" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="E68" s="10" t="s">
+        <v>175</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>381</v>
       </c>
-      <c r="G68" s="8" t="s">
-        <v>223</v>
-      </c>
-      <c r="H68" s="7" t="s">
-        <v>335</v>
-      </c>
-      <c r="I68" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J68" s="7">
+      <c r="G68" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="H68" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="I68" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J68" s="9">
         <v>2</v>
       </c>
-      <c r="K68" s="7"/>
+      <c r="K68" s="9"/>
     </row>
     <row r="69" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B69) - ROW($B$2)</f>
         <v>67</v>
       </c>
-      <c r="C69" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="D69" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="E69" s="10" t="s">
-        <v>174</v>
+      <c r="C69" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D69" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E69" s="8" t="s">
+        <v>176</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>381</v>
       </c>
-      <c r="G69" s="10" t="s">
-        <v>224</v>
-      </c>
-      <c r="H69" s="9" t="s">
-        <v>336</v>
-      </c>
-      <c r="I69" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J69" s="9">
-        <v>1</v>
-      </c>
-      <c r="K69" s="9"/>
+      <c r="G69" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="H69" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="I69" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J69" s="7">
+        <v>1</v>
+      </c>
+      <c r="K69" s="7"/>
     </row>
     <row r="70" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
       <c r="B70" s="11">
-        <f>ROW(B70) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>68</v>
       </c>
-      <c r="C70" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D70" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="E70" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="F70" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="G70" s="8" t="s">
+      <c r="C70" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="E70" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="F70" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="G70" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="H70" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="I70" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J70" s="7">
-        <v>1</v>
-      </c>
-      <c r="K70" s="7"/>
+      <c r="H70" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="I70" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J70" s="9">
+        <v>1</v>
+      </c>
+      <c r="K70" s="9"/>
     </row>
     <row r="71" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
       <c r="B71" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B71) - ROW($B$2)</f>
         <v>69</v>
       </c>
-      <c r="C71" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D71" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="E71" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="F71" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="G71" s="10" t="s">
+      <c r="C71" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D71" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E71" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="F71" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="G71" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="H71" s="9" t="s">
-        <v>332</v>
-      </c>
-      <c r="I71" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J71" s="9">
-        <v>1</v>
-      </c>
-      <c r="K71" s="9"/>
+      <c r="H71" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="I71" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J71" s="7">
+        <v>1</v>
+      </c>
+      <c r="K71" s="7"/>
     </row>
     <row r="72" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
       <c r="B72" s="11">
-        <f>ROW(B72) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="C72" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D72" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="E72" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="F72" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="G72" s="8" t="s">
+      <c r="C72" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="E72" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="F72" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="G72" s="10" t="s">
         <v>295</v>
       </c>
-      <c r="H72" s="7" t="s">
-        <v>319</v>
-      </c>
-      <c r="I72" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J72" s="7">
-        <v>1</v>
-      </c>
-      <c r="K72" s="7"/>
+      <c r="H72" s="9" t="s">
+        <v>320</v>
+      </c>
+      <c r="I72" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J72" s="9">
+        <v>1</v>
+      </c>
+      <c r="K72" s="9"/>
     </row>
     <row r="73" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
       <c r="B73" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B73) - ROW($B$2)</f>
         <v>71</v>
       </c>
-      <c r="C73" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D73" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="E73" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="F73" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="G73" s="10" t="s">
+      <c r="C73" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D73" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E73" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="F73" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="G73" s="8" t="s">
         <v>296</v>
       </c>
-      <c r="H73" s="9" t="s">
-        <v>319</v>
-      </c>
-      <c r="I73" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J73" s="9">
-        <v>1</v>
-      </c>
-      <c r="K73" s="9"/>
+      <c r="H73" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="I73" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J73" s="7">
+        <v>1</v>
+      </c>
+      <c r="K73" s="7"/>
     </row>
     <row r="74" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
       <c r="B74" s="11">
-        <f>ROW(B74) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>72</v>
       </c>
-      <c r="C74" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D74" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="E74" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="F74" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="G74" s="8" t="s">
+      <c r="C74" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D74" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E74" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="F74" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="G74" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="H74" s="7" t="s">
-        <v>337</v>
-      </c>
-      <c r="I74" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J74" s="7">
-        <v>1</v>
-      </c>
-      <c r="K74" s="7"/>
+      <c r="H74" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="I74" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J74" s="9">
+        <v>1</v>
+      </c>
+      <c r="K74" s="9"/>
     </row>
     <row r="75" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B75) - ROW($B$2)</f>
         <v>73</v>
       </c>
-      <c r="C75" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D75" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="E75" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="F75" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="G75" s="10" t="s">
+      <c r="C75" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D75" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="E75" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="F75" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="G75" s="8" t="s">
         <v>298</v>
       </c>
-      <c r="H75" s="9" t="s">
-        <v>319</v>
-      </c>
-      <c r="I75" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J75" s="9">
-        <v>1</v>
-      </c>
-      <c r="K75" s="9"/>
+      <c r="H75" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="I75" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J75" s="7">
+        <v>1</v>
+      </c>
+      <c r="K75" s="7"/>
     </row>
     <row r="76" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
       <c r="B76" s="11">
-        <f>ROW(B76) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>74</v>
       </c>
-      <c r="C76" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="D76" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="E76" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="F76" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="G76" s="8" t="s">
+      <c r="C76" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E76" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="F76" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="G76" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="H76" s="7" t="s">
-        <v>321</v>
-      </c>
-      <c r="I76" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J76" s="7">
-        <v>1</v>
-      </c>
-      <c r="K76" s="7"/>
+      <c r="H76" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="I76" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J76" s="9">
+        <v>1</v>
+      </c>
+      <c r="K76" s="9"/>
     </row>
     <row r="77" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
       <c r="B77" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B77) - ROW($B$2)</f>
         <v>75</v>
       </c>
-      <c r="C77" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D77" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="E77" s="10" t="s">
-        <v>182</v>
-      </c>
-      <c r="F77" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="G77" s="10" t="s">
+      <c r="C77" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D77" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E77" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="F77" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="G77" s="8" t="s">
         <v>300</v>
       </c>
-      <c r="H77" s="9" t="s">
-        <v>332</v>
-      </c>
-      <c r="I77" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J77" s="9">
-        <v>1</v>
-      </c>
-      <c r="K77" s="9"/>
+      <c r="H77" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="I77" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J77" s="7">
+        <v>1</v>
+      </c>
+      <c r="K77" s="7"/>
     </row>
     <row r="78" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
       <c r="B78" s="11">
-        <f>ROW(B78) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>76</v>
       </c>
-      <c r="C78" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D78" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="E78" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="F78" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="G78" s="8" t="s">
+      <c r="C78" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D78" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E78" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="F78" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="G78" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="H78" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="I78" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J78" s="7">
-        <v>1</v>
-      </c>
-      <c r="K78" s="7"/>
+      <c r="H78" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="I78" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J78" s="9">
+        <v>1</v>
+      </c>
+      <c r="K78" s="9"/>
     </row>
     <row r="79" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
       <c r="B79" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B79) - ROW($B$2)</f>
         <v>77</v>
       </c>
-      <c r="C79" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D79" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="E79" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="F79" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="G79" s="10" t="s">
+      <c r="C79" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D79" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E79" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="F79" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="G79" s="8" t="s">
         <v>302</v>
       </c>
-      <c r="H79" s="9" t="s">
-        <v>332</v>
-      </c>
-      <c r="I79" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J79" s="9">
+      <c r="H79" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="I79" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J79" s="7">
         <v>16</v>
       </c>
-      <c r="K79" s="9"/>
+      <c r="K79" s="7"/>
     </row>
     <row r="80" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
       <c r="B80" s="11">
-        <f>ROW(B80) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>78</v>
       </c>
-      <c r="C80" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D80" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E80" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="F80" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="G80" s="8" t="s">
+      <c r="C80" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D80" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="E80" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="F80" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="G80" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="H80" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="I80" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J80" s="7">
+      <c r="H80" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="I80" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J80" s="9">
         <v>4</v>
       </c>
-      <c r="K80" s="7"/>
+      <c r="K80" s="9"/>
     </row>
     <row r="81" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
       <c r="B81" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B81) - ROW($B$2)</f>
         <v>79</v>
       </c>
-      <c r="C81" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D81" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="E81" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="F81" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="G81" s="10" t="s">
+      <c r="C81" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E81" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="F81" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="G81" s="8" t="s">
         <v>304</v>
       </c>
-      <c r="H81" s="9" t="s">
-        <v>332</v>
-      </c>
-      <c r="I81" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="J81" s="9">
-        <v>1</v>
-      </c>
-      <c r="K81" s="9"/>
+      <c r="H81" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="I81" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J81" s="7">
+        <v>1</v>
+      </c>
+      <c r="K81" s="7"/>
     </row>
     <row r="82" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1"/>
       <c r="B82" s="11">
-        <f>ROW(B82) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="C82" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D82" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="E82" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="F82" s="7" t="s">
-        <v>235</v>
-      </c>
-      <c r="G82" s="8" t="s">
+      <c r="C82" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D82" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="E82" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="F82" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="G82" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="H82" s="7" t="s">
-        <v>338</v>
-      </c>
-      <c r="I82" s="8" t="s">
-        <v>374</v>
-      </c>
-      <c r="J82" s="7">
-        <v>1</v>
-      </c>
-      <c r="K82" s="7"/>
+      <c r="H82" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="I82" s="10" t="s">
+        <v>375</v>
+      </c>
+      <c r="J82" s="9">
+        <v>1</v>
+      </c>
+      <c r="K82" s="9"/>
     </row>
     <row r="83" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1"/>
       <c r="B83" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B83) - ROW($B$2)</f>
         <v>81</v>
       </c>
-      <c r="C83" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D83" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="E83" s="10" t="s">
-        <v>187</v>
+      <c r="C83" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D83" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E83" s="8" t="s">
+        <v>189</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>381</v>
       </c>
-      <c r="G83" s="10" t="s">
+      <c r="G83" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="H83" s="9" t="s">
-        <v>339</v>
-      </c>
-      <c r="I83" s="10" t="s">
-        <v>375</v>
-      </c>
-      <c r="J83" s="9">
-        <v>1</v>
-      </c>
-      <c r="K83" s="9"/>
+      <c r="H83" s="7" t="s">
+        <v>340</v>
+      </c>
+      <c r="I83" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="J83" s="7">
+        <v>1</v>
+      </c>
+      <c r="K83" s="7"/>
+    </row>
+    <row r="84" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B84" s="11">
+        <f t="shared" si="0"/>
+        <v>82</v>
+      </c>
+      <c r="C84" s="13" t="s">
+        <v>384</v>
+      </c>
+      <c r="D84" s="9" t="s">
+        <v>385</v>
+      </c>
+      <c r="E84" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="F84" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="G84" s="10" t="s">
+        <v>392</v>
+      </c>
+      <c r="H84" s="9" t="s">
+        <v>323</v>
+      </c>
+      <c r="I84" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J84" s="9">
+        <v>1</v>
+      </c>
+      <c r="K84" s="9"/>
+    </row>
+    <row r="85" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B85" s="11">
+        <f>ROW(B85) - ROW($B$2)</f>
+        <v>83</v>
+      </c>
+      <c r="C85" s="13" t="s">
+        <v>384</v>
+      </c>
+      <c r="D85" s="7" t="s">
+        <v>386</v>
+      </c>
+      <c r="E85" s="8" t="s">
+        <v>391</v>
+      </c>
+      <c r="F85" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="G85" s="8" t="s">
+        <v>390</v>
+      </c>
+      <c r="H85" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I85" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J85" s="7">
+        <v>2</v>
+      </c>
+      <c r="K85" s="7"/>
+    </row>
+    <row r="86" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B86" s="11">
+        <f t="shared" ref="B86" si="1">ROW(B86) - ROW($B$2)</f>
+        <v>84</v>
+      </c>
+      <c r="C86" s="13" t="s">
+        <v>384</v>
+      </c>
+      <c r="D86" s="9" t="s">
+        <v>387</v>
+      </c>
+      <c r="E86" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="F86" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="G86" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="H86" s="9" t="s">
+        <v>380</v>
+      </c>
+      <c r="I86" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="J86" s="9" t="s">
+        <v>380</v>
+      </c>
+      <c r="K86" s="14" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B87" s="11">
+        <f>ROW(B87) - ROW($B$2)</f>
+        <v>85</v>
+      </c>
+      <c r="C87" s="13" t="s">
+        <v>384</v>
+      </c>
+      <c r="D87" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="E87" s="8" t="s">
+        <v>395</v>
+      </c>
+      <c r="F87" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="G87" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="H87" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="I87" s="8" t="s">
+        <v>380</v>
+      </c>
+      <c r="J87" s="7">
+        <v>1</v>
+      </c>
+      <c r="K87" s="19" t="s">
+        <v>383</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
#52 R130, R131 Added in Client BOM.
</commit_message>
<xml_diff>
--- a/Design Files/Stepper-Driver-v2.0/BOM/Client-BOM-Stepper-Driver-v2.0.xlsx
+++ b/Design Files/Stepper-Driver-v2.0/BOM/Client-BOM-Stepper-Driver-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="395">
   <si>
     <t>#</t>
   </si>
@@ -1192,6 +1192,18 @@
   </si>
   <si>
     <t>TC2030-CTX</t>
+  </si>
+  <si>
+    <t>R130, R131</t>
+  </si>
+  <si>
+    <t>RES 560 OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-07560RL</t>
+  </si>
+  <si>
+    <t>560R</t>
   </si>
 </sst>
 </file>
@@ -1698,7 +1710,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K86"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1711,6 +1723,8 @@
     <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.140625" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1794,7 +1808,7 @@
     <row r="4" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B83" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B84" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -3810,640 +3824,671 @@
     <row r="67" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="11">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B67" si="1">ROW(B67) - ROW($B$2)</f>
         <v>65</v>
       </c>
       <c r="C67" s="13" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>92</v>
+        <v>391</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>173</v>
+        <v>392</v>
       </c>
       <c r="F67" s="9" t="s">
-        <v>377</v>
+        <v>218</v>
       </c>
       <c r="G67" s="10" t="s">
-        <v>222</v>
+        <v>393</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>332</v>
+        <v>307</v>
       </c>
       <c r="I67" s="10" t="s">
-        <v>376</v>
+        <v>394</v>
       </c>
       <c r="J67" s="9">
         <v>2</v>
       </c>
       <c r="K67" s="9"/>
     </row>
-    <row r="68" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="11">
-        <f>ROW(B68) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>66</v>
       </c>
-      <c r="C68" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D68" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="E68" s="8" t="s">
-        <v>174</v>
+      <c r="C68" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D68" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="E68" s="10" t="s">
+        <v>173</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>377</v>
       </c>
-      <c r="G68" s="8" t="s">
-        <v>223</v>
-      </c>
-      <c r="H68" s="7" t="s">
-        <v>333</v>
+      <c r="G68" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H68" s="9" t="s">
+        <v>332</v>
       </c>
       <c r="I68" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J68" s="7">
-        <v>1</v>
-      </c>
-      <c r="K68" s="7"/>
-    </row>
-    <row r="69" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J68" s="9">
+        <v>2</v>
+      </c>
+      <c r="K68" s="9"/>
+    </row>
+    <row r="69" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B69) - ROW($B$2)</f>
         <v>67</v>
       </c>
-      <c r="C69" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D69" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="E69" s="10" t="s">
-        <v>175</v>
+      <c r="C69" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D69" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="E69" s="8" t="s">
+        <v>174</v>
       </c>
       <c r="F69" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="G69" s="10" t="s">
-        <v>290</v>
-      </c>
-      <c r="H69" s="9" t="s">
-        <v>329</v>
+        <v>377</v>
+      </c>
+      <c r="G69" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="H69" s="7" t="s">
+        <v>333</v>
       </c>
       <c r="I69" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J69" s="9">
-        <v>1</v>
-      </c>
-      <c r="K69" s="9"/>
-    </row>
-    <row r="70" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J69" s="7">
+        <v>1</v>
+      </c>
+      <c r="K69" s="7"/>
+    </row>
+    <row r="70" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
       <c r="B70" s="11">
-        <f>ROW(B70) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>68</v>
       </c>
-      <c r="C70" s="12" t="s">
+      <c r="C70" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D70" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="E70" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="F70" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="G70" s="8" t="s">
-        <v>291</v>
-      </c>
-      <c r="H70" s="7" t="s">
+      <c r="D70" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E70" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="F70" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="G70" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="H70" s="9" t="s">
         <v>329</v>
       </c>
       <c r="I70" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J70" s="7">
-        <v>1</v>
-      </c>
-      <c r="K70" s="7"/>
+      <c r="J70" s="9">
+        <v>1</v>
+      </c>
+      <c r="K70" s="9"/>
     </row>
     <row r="71" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
       <c r="B71" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B71) - ROW($B$2)</f>
         <v>69</v>
       </c>
-      <c r="C71" s="13" t="s">
+      <c r="C71" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D71" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="E71" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="F71" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="G71" s="10" t="s">
-        <v>292</v>
-      </c>
-      <c r="H71" s="9" t="s">
-        <v>317</v>
+      <c r="D71" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E71" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="F71" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="G71" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="H71" s="7" t="s">
+        <v>329</v>
       </c>
       <c r="I71" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J71" s="9">
-        <v>1</v>
-      </c>
-      <c r="K71" s="9"/>
+      <c r="J71" s="7">
+        <v>1</v>
+      </c>
+      <c r="K71" s="7"/>
     </row>
     <row r="72" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
       <c r="B72" s="11">
-        <f>ROW(B72) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="C72" s="12" t="s">
+      <c r="C72" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D72" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="E72" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="F72" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="G72" s="8" t="s">
-        <v>293</v>
-      </c>
-      <c r="H72" s="7" t="s">
+      <c r="D72" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="E72" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="F72" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="G72" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="H72" s="9" t="s">
         <v>317</v>
       </c>
       <c r="I72" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J72" s="7">
-        <v>1</v>
-      </c>
-      <c r="K72" s="7"/>
+      <c r="J72" s="9">
+        <v>1</v>
+      </c>
+      <c r="K72" s="9"/>
     </row>
     <row r="73" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
       <c r="B73" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B73) - ROW($B$2)</f>
         <v>71</v>
       </c>
-      <c r="C73" s="13" t="s">
+      <c r="C73" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D73" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="E73" s="10" t="s">
-        <v>179</v>
-      </c>
-      <c r="F73" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="G73" s="10" t="s">
-        <v>294</v>
-      </c>
-      <c r="H73" s="9" t="s">
-        <v>334</v>
+      <c r="D73" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E73" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="F73" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="G73" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="H73" s="7" t="s">
+        <v>317</v>
       </c>
       <c r="I73" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J73" s="9">
-        <v>1</v>
-      </c>
-      <c r="K73" s="9"/>
+      <c r="J73" s="7">
+        <v>1</v>
+      </c>
+      <c r="K73" s="7"/>
     </row>
     <row r="74" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
       <c r="B74" s="11">
-        <f>ROW(B74) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>72</v>
       </c>
-      <c r="C74" s="12" t="s">
+      <c r="C74" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D74" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="E74" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="F74" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="G74" s="8" t="s">
-        <v>295</v>
-      </c>
-      <c r="H74" s="7" t="s">
-        <v>317</v>
+      <c r="D74" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E74" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="F74" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="G74" s="10" t="s">
+        <v>294</v>
+      </c>
+      <c r="H74" s="9" t="s">
+        <v>334</v>
       </c>
       <c r="I74" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J74" s="7">
-        <v>1</v>
-      </c>
-      <c r="K74" s="7"/>
-    </row>
-    <row r="75" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J74" s="9">
+        <v>1</v>
+      </c>
+      <c r="K74" s="9"/>
+    </row>
+    <row r="75" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B75) - ROW($B$2)</f>
         <v>73</v>
       </c>
-      <c r="C75" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="D75" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="E75" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="F75" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="G75" s="10" t="s">
-        <v>296</v>
-      </c>
-      <c r="H75" s="9" t="s">
-        <v>319</v>
+      <c r="C75" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D75" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E75" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="F75" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="G75" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="H75" s="7" t="s">
+        <v>317</v>
       </c>
       <c r="I75" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J75" s="9">
-        <v>1</v>
-      </c>
-      <c r="K75" s="9"/>
-    </row>
-    <row r="76" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J75" s="7">
+        <v>1</v>
+      </c>
+      <c r="K75" s="7"/>
+    </row>
+    <row r="76" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
       <c r="B76" s="11">
-        <f>ROW(B76) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>74</v>
       </c>
-      <c r="C76" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D76" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="E76" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="F76" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="G76" s="8" t="s">
-        <v>297</v>
-      </c>
-      <c r="H76" s="7" t="s">
-        <v>329</v>
+      <c r="C76" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="E76" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="F76" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="G76" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="H76" s="9" t="s">
+        <v>319</v>
       </c>
       <c r="I76" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J76" s="7">
-        <v>1</v>
-      </c>
-      <c r="K76" s="7"/>
+      <c r="J76" s="9">
+        <v>1</v>
+      </c>
+      <c r="K76" s="9"/>
     </row>
     <row r="77" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
       <c r="B77" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B77) - ROW($B$2)</f>
         <v>75</v>
       </c>
-      <c r="C77" s="13" t="s">
+      <c r="C77" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D77" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="E77" s="10" t="s">
+      <c r="D77" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E77" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="F77" s="9" t="s">
+      <c r="F77" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="G77" s="10" t="s">
-        <v>298</v>
-      </c>
-      <c r="H77" s="9" t="s">
+      <c r="G77" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="H77" s="7" t="s">
         <v>329</v>
       </c>
       <c r="I77" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J77" s="9">
-        <v>1</v>
-      </c>
-      <c r="K77" s="9"/>
-    </row>
-    <row r="78" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J77" s="7">
+        <v>1</v>
+      </c>
+      <c r="K77" s="7"/>
+    </row>
+    <row r="78" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
       <c r="B78" s="11">
-        <f>ROW(B78) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>76</v>
       </c>
-      <c r="C78" s="12" t="s">
+      <c r="C78" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D78" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E78" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="F78" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="G78" s="8" t="s">
-        <v>299</v>
-      </c>
-      <c r="H78" s="7" t="s">
+      <c r="D78" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="E78" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="F78" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="G78" s="10" t="s">
+        <v>298</v>
+      </c>
+      <c r="H78" s="9" t="s">
         <v>329</v>
       </c>
       <c r="I78" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J78" s="7">
-        <v>16</v>
-      </c>
-      <c r="K78" s="7"/>
-    </row>
-    <row r="79" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J78" s="9">
+        <v>1</v>
+      </c>
+      <c r="K78" s="9"/>
+    </row>
+    <row r="79" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
       <c r="B79" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B79) - ROW($B$2)</f>
         <v>77</v>
       </c>
-      <c r="C79" s="13" t="s">
+      <c r="C79" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D79" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="E79" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="F79" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="G79" s="10" t="s">
-        <v>300</v>
-      </c>
-      <c r="H79" s="9" t="s">
+      <c r="D79" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E79" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="F79" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="G79" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="H79" s="7" t="s">
         <v>329</v>
       </c>
       <c r="I79" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J79" s="9">
-        <v>4</v>
-      </c>
-      <c r="K79" s="9"/>
+      <c r="J79" s="7">
+        <v>16</v>
+      </c>
+      <c r="K79" s="7"/>
     </row>
     <row r="80" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
       <c r="B80" s="11">
-        <f>ROW(B80) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>78</v>
       </c>
-      <c r="C80" s="12" t="s">
+      <c r="C80" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D80" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="E80" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="F80" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="G80" s="8" t="s">
-        <v>301</v>
-      </c>
-      <c r="H80" s="7" t="s">
+      <c r="D80" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="E80" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="F80" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="G80" s="10" t="s">
+        <v>300</v>
+      </c>
+      <c r="H80" s="9" t="s">
         <v>329</v>
       </c>
       <c r="I80" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J80" s="7">
-        <v>1</v>
-      </c>
-      <c r="K80" s="7"/>
-    </row>
-    <row r="81" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J80" s="9">
+        <v>4</v>
+      </c>
+      <c r="K80" s="9"/>
+    </row>
+    <row r="81" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
       <c r="B81" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B81) - ROW($B$2)</f>
         <v>79</v>
       </c>
-      <c r="C81" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="D81" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="E81" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="F81" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="G81" s="10" t="s">
-        <v>302</v>
-      </c>
-      <c r="H81" s="9" t="s">
-        <v>335</v>
+      <c r="C81" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E81" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="F81" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="G81" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="H81" s="7" t="s">
+        <v>329</v>
       </c>
       <c r="I81" s="10" t="s">
-        <v>371</v>
-      </c>
-      <c r="J81" s="9">
-        <v>1</v>
-      </c>
-      <c r="K81" s="9"/>
-    </row>
-    <row r="82" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>376</v>
+      </c>
+      <c r="J81" s="7">
+        <v>1</v>
+      </c>
+      <c r="K81" s="7"/>
+    </row>
+    <row r="82" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1"/>
       <c r="B82" s="11">
-        <f>ROW(B82) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>80</v>
       </c>
       <c r="C82" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D82" s="7" t="s">
+      <c r="D82" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="E82" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="F82" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="G82" s="10" t="s">
+        <v>302</v>
+      </c>
+      <c r="H82" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="I82" s="10" t="s">
+        <v>371</v>
+      </c>
+      <c r="J82" s="9">
+        <v>1</v>
+      </c>
+      <c r="K82" s="9"/>
+    </row>
+    <row r="83" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B83" s="11">
+        <f>ROW(B83) - ROW($B$2)</f>
+        <v>81</v>
+      </c>
+      <c r="C83" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D83" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="E82" s="8" t="s">
+      <c r="E83" s="8" t="s">
         <v>187</v>
-      </c>
-      <c r="F82" s="9" t="s">
-        <v>377</v>
-      </c>
-      <c r="G82" s="8" t="s">
-        <v>303</v>
-      </c>
-      <c r="H82" s="7" t="s">
-        <v>336</v>
-      </c>
-      <c r="I82" s="8" t="s">
-        <v>372</v>
-      </c>
-      <c r="J82" s="7">
-        <v>1</v>
-      </c>
-      <c r="K82" s="7"/>
-    </row>
-    <row r="83" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="11">
-        <f t="shared" si="0"/>
-        <v>81</v>
-      </c>
-      <c r="C83" s="13" t="s">
-        <v>379</v>
-      </c>
-      <c r="D83" s="9" t="s">
-        <v>380</v>
-      </c>
-      <c r="E83" s="10" t="s">
-        <v>387</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>377</v>
       </c>
-      <c r="G83" s="10" t="s">
-        <v>386</v>
-      </c>
-      <c r="H83" s="9" t="s">
-        <v>320</v>
-      </c>
-      <c r="I83" s="10" t="s">
-        <v>376</v>
-      </c>
-      <c r="J83" s="9">
-        <v>1</v>
-      </c>
-      <c r="K83" s="9"/>
+      <c r="G83" s="8" t="s">
+        <v>303</v>
+      </c>
+      <c r="H83" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="I83" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="J83" s="7">
+        <v>1</v>
+      </c>
+      <c r="K83" s="7"/>
     </row>
     <row r="84" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B84" s="11">
-        <f>ROW(B84) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>82</v>
       </c>
       <c r="C84" s="13" t="s">
         <v>379</v>
       </c>
-      <c r="D84" s="7" t="s">
-        <v>381</v>
-      </c>
-      <c r="E84" s="8" t="s">
-        <v>385</v>
+      <c r="D84" s="9" t="s">
+        <v>380</v>
+      </c>
+      <c r="E84" s="10" t="s">
+        <v>387</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>377</v>
       </c>
-      <c r="G84" s="8" t="s">
-        <v>384</v>
-      </c>
-      <c r="H84" s="7" t="s">
-        <v>324</v>
+      <c r="G84" s="10" t="s">
+        <v>386</v>
+      </c>
+      <c r="H84" s="9" t="s">
+        <v>320</v>
       </c>
       <c r="I84" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J84" s="7">
-        <v>2</v>
-      </c>
-      <c r="K84" s="7"/>
-    </row>
-    <row r="85" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J84" s="9">
+        <v>1</v>
+      </c>
+      <c r="K84" s="9"/>
+    </row>
+    <row r="85" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B85" s="11">
-        <f t="shared" ref="B85" si="1">ROW(B85) - ROW($B$2)</f>
+        <f>ROW(B85) - ROW($B$2)</f>
         <v>83</v>
       </c>
       <c r="C85" s="13" t="s">
         <v>379</v>
       </c>
-      <c r="D85" s="9" t="s">
-        <v>382</v>
-      </c>
-      <c r="E85" s="10" t="s">
-        <v>376</v>
+      <c r="D85" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="E85" s="8" t="s">
+        <v>385</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>377</v>
       </c>
-      <c r="G85" s="10" t="s">
-        <v>376</v>
-      </c>
-      <c r="H85" s="9" t="s">
-        <v>376</v>
+      <c r="G85" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="H85" s="7" t="s">
+        <v>324</v>
       </c>
       <c r="I85" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="J85" s="9" t="s">
-        <v>376</v>
-      </c>
-      <c r="K85" s="14" t="s">
-        <v>388</v>
-      </c>
+      <c r="J85" s="7">
+        <v>2</v>
+      </c>
+      <c r="K85" s="7"/>
     </row>
     <row r="86" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B86" s="11">
-        <f>ROW(B86) - ROW($B$2)</f>
+        <f t="shared" ref="B86" si="2">ROW(B86) - ROW($B$2)</f>
         <v>84</v>
       </c>
       <c r="C86" s="13" t="s">
         <v>379</v>
       </c>
-      <c r="D86" s="7" t="s">
-        <v>383</v>
-      </c>
-      <c r="E86" s="8" t="s">
-        <v>389</v>
+      <c r="D86" s="9" t="s">
+        <v>382</v>
+      </c>
+      <c r="E86" s="10" t="s">
+        <v>376</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>377</v>
       </c>
-      <c r="G86" s="8" t="s">
+      <c r="G86" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="H86" s="9" t="s">
+        <v>376</v>
+      </c>
+      <c r="I86" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="J86" s="9" t="s">
+        <v>376</v>
+      </c>
+      <c r="K86" s="14" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B87" s="11">
+        <f>ROW(B87) - ROW($B$2)</f>
+        <v>85</v>
+      </c>
+      <c r="C87" s="13" t="s">
+        <v>379</v>
+      </c>
+      <c r="D87" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="E87" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="F87" s="9" t="s">
+        <v>377</v>
+      </c>
+      <c r="G87" s="8" t="s">
         <v>390</v>
       </c>
-      <c r="H86" s="7" t="s">
-        <v>376</v>
-      </c>
-      <c r="I86" s="8" t="s">
-        <v>376</v>
-      </c>
-      <c r="J86" s="7">
-        <v>1</v>
-      </c>
-      <c r="K86" s="15" t="s">
+      <c r="H87" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="I87" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="J87" s="7">
+        <v>1</v>
+      </c>
+      <c r="K87" s="15" t="s">
         <v>378</v>
       </c>
     </row>

</xml_diff>